<commit_message>
typo in header fixed
</commit_message>
<xml_diff>
--- a/resources/vega_models_withclasses.xlsx
+++ b/resources/vega_models_withclasses.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="1034">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="1034">
   <si>
     <t>Key</t>
   </si>
@@ -2626,9 +2626,6 @@
     <t>PMT</t>
   </si>
   <si>
-    <t>ENDPOINT_CATEORIES</t>
-  </si>
-  <si>
     <t>EC_FISHTOX_SECTION</t>
   </si>
   <si>
@@ -3122,6 +3119,9 @@
   </si>
   <si>
     <t>Endocrine_disruption</t>
+  </si>
+  <si>
+    <t>ENDPOINT_CATEGORY</t>
   </si>
 </sst>
 </file>
@@ -3705,15 +3705,9 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:N114" totalsRowShown="0">
-  <autoFilter ref="A1:N114">
-    <filterColumn colId="11">
-      <filters>
-        <filter val="ED_(human)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <sortState ref="A2:N114">
-    <sortCondition ref="L1:L114"/>
+  <autoFilter ref="A1:N114"/>
+  <sortState ref="A34:N50">
+    <sortCondition ref="M1:M114"/>
   </sortState>
   <tableColumns count="14">
     <tableColumn id="1" name="Key"/>
@@ -3728,7 +3722,7 @@
     <tableColumn id="10" name="ADItemsName"/>
     <tableColumn id="11" name="ResultsName"/>
     <tableColumn id="12" name="SSbD" dataDxfId="0"/>
-    <tableColumn id="13" name="ENDPOINT_CATEORIES"/>
+    <tableColumn id="13" name="ENDPOINT_CATEGORY"/>
     <tableColumn id="14" name="Column1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4011,7 +4005,7 @@
     <col min="10" max="10" width="14.6640625" customWidth="1"/>
     <col min="11" max="11" width="66.77734375" customWidth="1"/>
     <col min="12" max="12" width="25.77734375" customWidth="1"/>
-    <col min="13" max="13" width="15.21875" customWidth="1"/>
+    <col min="13" max="13" width="35.33203125" customWidth="1"/>
     <col min="14" max="14" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4053,13 +4047,13 @@
         <v>866</v>
       </c>
       <c r="M1" t="s">
-        <v>868</v>
+        <v>1033</v>
       </c>
       <c r="N1" t="s">
-        <v>870</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -4094,13 +4088,13 @@
         <v>21</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="M2" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -4132,13 +4126,13 @@
         <v>30</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="M3" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -4173,13 +4167,13 @@
         <v>38</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="M4" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -4214,13 +4208,13 @@
         <v>45</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M5" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>197</v>
       </c>
@@ -4255,13 +4249,13 @@
         <v>204</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="M6" t="s">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>205</v>
       </c>
@@ -4297,13 +4291,13 @@
         <v>212</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="M7" t="s">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>213</v>
       </c>
@@ -4338,13 +4332,13 @@
         <v>204</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="M8" t="s">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>219</v>
       </c>
@@ -4380,13 +4374,13 @@
         <v>212</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="M9" t="s">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>226</v>
       </c>
@@ -4421,13 +4415,13 @@
         <v>232</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M10" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>289</v>
       </c>
@@ -4463,13 +4457,13 @@
         <v>212</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M11" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>296</v>
       </c>
@@ -4504,13 +4498,13 @@
         <v>303</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M12" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>304</v>
       </c>
@@ -4546,13 +4540,13 @@
         <v>310</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M13" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>311</v>
       </c>
@@ -4584,13 +4578,13 @@
         <v>318</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M14" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>319</v>
       </c>
@@ -4626,13 +4620,13 @@
         <v>325</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M15" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>326</v>
       </c>
@@ -4667,13 +4661,13 @@
         <v>332</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M16" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>333</v>
       </c>
@@ -4708,13 +4702,13 @@
         <v>340</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M17" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>341</v>
       </c>
@@ -4749,13 +4743,13 @@
         <v>45</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M18" t="s">
-        <v>874</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>355</v>
       </c>
@@ -4790,13 +4784,13 @@
         <v>303</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M19" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>499</v>
       </c>
@@ -4828,13 +4822,13 @@
         <v>506</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M20" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>507</v>
       </c>
@@ -4863,13 +4857,13 @@
         <v>513</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M21" t="s">
-        <v>874</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>844</v>
       </c>
@@ -4898,13 +4892,13 @@
         <v>850</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="M22" t="s">
-        <v>1025</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>858</v>
       </c>
@@ -4939,13 +4933,13 @@
         <v>865</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="M23" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>106</v>
       </c>
@@ -4977,13 +4971,13 @@
         <v>114</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M24" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>124</v>
       </c>
@@ -5015,13 +5009,13 @@
         <v>132</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M25" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>115</v>
       </c>
@@ -5053,13 +5047,13 @@
         <v>123</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M26" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>133</v>
       </c>
@@ -5091,13 +5085,13 @@
         <v>114</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M27" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>152</v>
       </c>
@@ -5129,13 +5123,13 @@
         <v>159</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M28" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>160</v>
       </c>
@@ -5170,13 +5164,13 @@
         <v>167</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M29" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>168</v>
       </c>
@@ -5208,13 +5202,13 @@
         <v>174</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M30" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>175</v>
       </c>
@@ -5249,13 +5243,13 @@
         <v>181</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M31" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>139</v>
       </c>
@@ -5287,13 +5281,13 @@
         <v>145</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M32" t="s">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>146</v>
       </c>
@@ -5325,10 +5319,10 @@
         <v>145</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="M33" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
@@ -5360,10 +5354,10 @@
         <v>54</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M34" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
@@ -5398,68 +5392,68 @@
         <v>62</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M35" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>347</v>
+        <v>575</v>
       </c>
       <c r="B36" t="s">
-        <v>348</v>
+        <v>576</v>
       </c>
       <c r="C36" t="s">
-        <v>349</v>
+        <v>577</v>
       </c>
       <c r="D36" t="s">
-        <v>350</v>
-      </c>
-      <c r="E36" t="s">
-        <v>35</v>
+        <v>578</v>
       </c>
       <c r="F36" t="s">
-        <v>351</v>
+        <v>579</v>
       </c>
       <c r="G36" t="s">
-        <v>352</v>
+        <v>263</v>
       </c>
       <c r="H36" t="s">
-        <v>353</v>
+        <v>580</v>
       </c>
       <c r="I36" t="s">
         <v>53</v>
       </c>
       <c r="K36" t="s">
-        <v>354</v>
+        <v>581</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
+      </c>
+      <c r="M36" t="s">
+        <v>1013</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>575</v>
+        <v>640</v>
       </c>
       <c r="B37" t="s">
-        <v>576</v>
+        <v>641</v>
       </c>
       <c r="C37" t="s">
-        <v>577</v>
+        <v>642</v>
       </c>
       <c r="D37" t="s">
-        <v>578</v>
+        <v>643</v>
       </c>
       <c r="F37" t="s">
-        <v>579</v>
+        <v>644</v>
       </c>
       <c r="G37" t="s">
         <v>263</v>
       </c>
       <c r="H37" t="s">
-        <v>580</v>
+        <v>645</v>
       </c>
       <c r="I37" t="s">
         <v>53</v>
@@ -5468,33 +5462,33 @@
         <v>581</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M37" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="B38" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="C38" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="D38" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="F38" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="G38" t="s">
         <v>263</v>
       </c>
       <c r="H38" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="I38" t="s">
         <v>53</v>
@@ -5503,33 +5497,33 @@
         <v>581</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M38" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>646</v>
+        <v>659</v>
       </c>
       <c r="B39" t="s">
-        <v>647</v>
+        <v>660</v>
       </c>
       <c r="C39" t="s">
-        <v>648</v>
+        <v>661</v>
       </c>
       <c r="D39" t="s">
-        <v>649</v>
+        <v>662</v>
       </c>
       <c r="F39" t="s">
-        <v>650</v>
+        <v>663</v>
       </c>
       <c r="G39" t="s">
         <v>263</v>
       </c>
       <c r="H39" t="s">
-        <v>651</v>
+        <v>664</v>
       </c>
       <c r="I39" t="s">
         <v>53</v>
@@ -5538,109 +5532,115 @@
         <v>581</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M39" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>659</v>
+        <v>632</v>
       </c>
       <c r="B40" t="s">
-        <v>660</v>
+        <v>633</v>
       </c>
       <c r="C40" t="s">
-        <v>661</v>
+        <v>634</v>
       </c>
       <c r="D40" t="s">
-        <v>662</v>
+        <v>635</v>
       </c>
       <c r="F40" t="s">
-        <v>663</v>
+        <v>636</v>
       </c>
       <c r="G40" t="s">
-        <v>263</v>
+        <v>637</v>
       </c>
       <c r="H40" t="s">
-        <v>664</v>
+        <v>638</v>
       </c>
       <c r="I40" t="s">
-        <v>53</v>
+        <v>19</v>
+      </c>
+      <c r="J40" t="s">
+        <v>29</v>
       </c>
       <c r="K40" t="s">
-        <v>581</v>
+        <v>639</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M40" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>632</v>
+        <v>652</v>
       </c>
       <c r="B41" t="s">
-        <v>633</v>
+        <v>653</v>
       </c>
       <c r="C41" t="s">
-        <v>634</v>
+        <v>654</v>
       </c>
       <c r="D41" t="s">
-        <v>635</v>
+        <v>655</v>
+      </c>
+      <c r="E41" t="s">
+        <v>35</v>
       </c>
       <c r="F41" t="s">
-        <v>636</v>
+        <v>656</v>
       </c>
       <c r="G41" t="s">
-        <v>637</v>
+        <v>17</v>
       </c>
       <c r="H41" t="s">
-        <v>638</v>
+        <v>657</v>
       </c>
       <c r="I41" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="J41" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="K41" t="s">
-        <v>639</v>
+        <v>658</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M41" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>652</v>
+        <v>441</v>
       </c>
       <c r="B42" t="s">
-        <v>653</v>
+        <v>442</v>
       </c>
       <c r="C42" t="s">
-        <v>654</v>
+        <v>443</v>
       </c>
       <c r="D42" t="s">
-        <v>655</v>
+        <v>444</v>
       </c>
       <c r="E42" t="s">
         <v>35</v>
       </c>
       <c r="F42" t="s">
-        <v>656</v>
+        <v>445</v>
       </c>
       <c r="G42" t="s">
         <v>17</v>
       </c>
       <c r="H42" t="s">
-        <v>657</v>
+        <v>446</v>
       </c>
       <c r="I42" t="s">
         <v>53</v>
@@ -5649,112 +5649,109 @@
         <v>20</v>
       </c>
       <c r="K42" t="s">
-        <v>658</v>
+        <v>447</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M42" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>441</v>
+        <v>828</v>
       </c>
       <c r="B43" t="s">
-        <v>442</v>
+        <v>829</v>
       </c>
       <c r="C43" t="s">
-        <v>443</v>
+        <v>830</v>
       </c>
       <c r="D43" t="s">
-        <v>444</v>
-      </c>
-      <c r="E43" t="s">
-        <v>35</v>
+        <v>831</v>
       </c>
       <c r="F43" t="s">
-        <v>445</v>
+        <v>832</v>
       </c>
       <c r="G43" t="s">
-        <v>17</v>
+        <v>833</v>
       </c>
       <c r="H43" t="s">
-        <v>446</v>
+        <v>834</v>
       </c>
       <c r="I43" t="s">
-        <v>53</v>
-      </c>
-      <c r="J43" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K43" t="s">
-        <v>447</v>
+        <v>835</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M43" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>665</v>
+        <v>347</v>
       </c>
       <c r="B44" t="s">
-        <v>666</v>
+        <v>348</v>
       </c>
       <c r="C44" t="s">
-        <v>667</v>
+        <v>349</v>
       </c>
       <c r="D44" t="s">
-        <v>668</v>
+        <v>350</v>
+      </c>
+      <c r="E44" t="s">
+        <v>35</v>
       </c>
       <c r="F44" t="s">
-        <v>669</v>
+        <v>351</v>
       </c>
       <c r="G44" t="s">
-        <v>670</v>
+        <v>352</v>
       </c>
       <c r="H44" t="s">
-        <v>671</v>
+        <v>353</v>
       </c>
       <c r="I44" t="s">
-        <v>19</v>
-      </c>
-      <c r="J44" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="K44" t="s">
-        <v>672</v>
+        <v>354</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
+      </c>
+      <c r="M44" t="s">
+        <v>1013</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>673</v>
+        <v>665</v>
       </c>
       <c r="B45" t="s">
-        <v>674</v>
+        <v>666</v>
       </c>
       <c r="C45" t="s">
-        <v>675</v>
+        <v>667</v>
       </c>
       <c r="D45" t="s">
-        <v>676</v>
+        <v>668</v>
       </c>
       <c r="F45" t="s">
-        <v>677</v>
+        <v>669</v>
       </c>
       <c r="G45" t="s">
-        <v>678</v>
+        <v>670</v>
       </c>
       <c r="H45" t="s">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="I45" t="s">
         <v>19</v>
@@ -5763,138 +5760,150 @@
         <v>61</v>
       </c>
       <c r="K45" t="s">
-        <v>680</v>
+        <v>672</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
+      </c>
+      <c r="M45" t="s">
+        <v>1013</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>681</v>
+        <v>673</v>
       </c>
       <c r="B46" t="s">
-        <v>682</v>
+        <v>674</v>
       </c>
       <c r="C46" t="s">
-        <v>683</v>
+        <v>675</v>
       </c>
       <c r="D46" t="s">
-        <v>684</v>
+        <v>676</v>
       </c>
       <c r="F46" t="s">
-        <v>685</v>
+        <v>677</v>
       </c>
       <c r="G46" t="s">
-        <v>263</v>
+        <v>678</v>
       </c>
       <c r="H46" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
       <c r="I46" t="s">
-        <v>113</v>
+        <v>19</v>
       </c>
       <c r="J46" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="K46" t="s">
-        <v>687</v>
+        <v>680</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
+      </c>
+      <c r="M46" t="s">
+        <v>1013</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>791</v>
+        <v>681</v>
       </c>
       <c r="B47" t="s">
-        <v>792</v>
+        <v>682</v>
       </c>
       <c r="C47" t="s">
-        <v>793</v>
+        <v>683</v>
       </c>
       <c r="D47" t="s">
-        <v>794</v>
+        <v>684</v>
       </c>
       <c r="F47" t="s">
-        <v>795</v>
+        <v>685</v>
       </c>
       <c r="G47" t="s">
-        <v>768</v>
+        <v>263</v>
       </c>
       <c r="H47" t="s">
-        <v>796</v>
+        <v>686</v>
       </c>
       <c r="I47" t="s">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="J47" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="K47" t="s">
-        <v>797</v>
+        <v>687</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
+      </c>
+      <c r="M47" t="s">
+        <v>1013</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="B48" t="s">
-        <v>799</v>
+        <v>792</v>
       </c>
       <c r="C48" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="D48" t="s">
-        <v>801</v>
+        <v>794</v>
       </c>
       <c r="F48" t="s">
-        <v>802</v>
+        <v>795</v>
       </c>
       <c r="G48" t="s">
-        <v>352</v>
+        <v>768</v>
       </c>
       <c r="H48" t="s">
-        <v>803</v>
+        <v>796</v>
       </c>
       <c r="I48" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="J48" t="s">
         <v>61</v>
       </c>
       <c r="K48" t="s">
-        <v>804</v>
+        <v>797</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
+      </c>
+      <c r="M48" t="s">
+        <v>1013</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>805</v>
+        <v>798</v>
       </c>
       <c r="B49" t="s">
-        <v>806</v>
+        <v>799</v>
       </c>
       <c r="C49" t="s">
-        <v>807</v>
+        <v>800</v>
       </c>
       <c r="D49" t="s">
-        <v>808</v>
+        <v>801</v>
       </c>
       <c r="F49" t="s">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="G49" t="s">
         <v>352</v>
       </c>
       <c r="H49" t="s">
-        <v>810</v>
+        <v>803</v>
       </c>
       <c r="I49" t="s">
         <v>19</v>
@@ -5903,48 +5912,54 @@
         <v>61</v>
       </c>
       <c r="K49" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
+      </c>
+      <c r="M49" t="s">
+        <v>1013</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>828</v>
+        <v>805</v>
       </c>
       <c r="B50" t="s">
-        <v>829</v>
+        <v>806</v>
       </c>
       <c r="C50" t="s">
-        <v>830</v>
+        <v>807</v>
       </c>
       <c r="D50" t="s">
-        <v>831</v>
+        <v>808</v>
       </c>
       <c r="F50" t="s">
-        <v>832</v>
+        <v>809</v>
       </c>
       <c r="G50" t="s">
-        <v>833</v>
+        <v>352</v>
       </c>
       <c r="H50" t="s">
-        <v>834</v>
+        <v>810</v>
       </c>
       <c r="I50" t="s">
         <v>19</v>
       </c>
+      <c r="J50" t="s">
+        <v>61</v>
+      </c>
       <c r="K50" t="s">
-        <v>835</v>
+        <v>811</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="M50" t="s">
-        <v>1014</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>266</v>
       </c>
@@ -5973,13 +5988,13 @@
         <v>273</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="M51" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>274</v>
       </c>
@@ -6011,13 +6026,13 @@
         <v>281</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="M52" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>282</v>
       </c>
@@ -6049,13 +6064,13 @@
         <v>288</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="M53" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>182</v>
       </c>
@@ -6087,13 +6102,13 @@
         <v>189</v>
       </c>
       <c r="L54" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M54" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>483</v>
       </c>
@@ -6125,13 +6140,13 @@
         <v>490</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M55" t="s">
-        <v>1010</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>491</v>
       </c>
@@ -6163,13 +6178,13 @@
         <v>498</v>
       </c>
       <c r="L56" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M56" t="s">
-        <v>1010</v>
-      </c>
-    </row>
-    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>514</v>
       </c>
@@ -6201,13 +6216,13 @@
         <v>521</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M57" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>529</v>
       </c>
@@ -6239,13 +6254,13 @@
         <v>521</v>
       </c>
       <c r="L58" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M58" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>522</v>
       </c>
@@ -6277,13 +6292,13 @@
         <v>521</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M59" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>537</v>
       </c>
@@ -6315,13 +6330,13 @@
         <v>544</v>
       </c>
       <c r="L60" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M60" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>545</v>
       </c>
@@ -6353,13 +6368,13 @@
         <v>553</v>
       </c>
       <c r="L61" s="3" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="M61" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>63</v>
       </c>
@@ -6394,13 +6409,13 @@
         <v>71</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M62" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>72</v>
       </c>
@@ -6435,13 +6450,13 @@
         <v>79</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M63" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>80</v>
       </c>
@@ -6476,13 +6491,13 @@
         <v>88</v>
       </c>
       <c r="L64" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M64" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="65" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>89</v>
       </c>
@@ -6517,13 +6532,13 @@
         <v>97</v>
       </c>
       <c r="L65" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M65" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="66" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>361</v>
       </c>
@@ -6558,13 +6573,13 @@
         <v>368</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M66" t="s">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="67" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>377</v>
       </c>
@@ -6599,13 +6614,13 @@
         <v>384</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M67" t="s">
-        <v>878</v>
-      </c>
-    </row>
-    <row r="68" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>385</v>
       </c>
@@ -6640,13 +6655,13 @@
         <v>393</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M68" t="s">
-        <v>879</v>
-      </c>
-    </row>
-    <row r="69" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>394</v>
       </c>
@@ -6681,13 +6696,13 @@
         <v>401</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M69" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="70" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>448</v>
       </c>
@@ -6719,13 +6734,13 @@
         <v>454</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M70" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="71" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>455</v>
       </c>
@@ -6757,13 +6772,13 @@
         <v>454</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M71" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="72" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>476</v>
       </c>
@@ -6795,13 +6810,13 @@
         <v>454</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M72" t="s">
-        <v>876</v>
-      </c>
-    </row>
-    <row r="73" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>688</v>
       </c>
@@ -6833,13 +6848,13 @@
         <v>695</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M73" t="s">
-        <v>875</v>
-      </c>
-    </row>
-    <row r="74" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>779</v>
       </c>
@@ -6874,13 +6889,13 @@
         <v>21</v>
       </c>
       <c r="L74" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M74" t="s">
-        <v>998</v>
-      </c>
-    </row>
-    <row r="75" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>785</v>
       </c>
@@ -6912,13 +6927,13 @@
         <v>30</v>
       </c>
       <c r="L75" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M75" t="s">
-        <v>998</v>
-      </c>
-    </row>
-    <row r="76" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>812</v>
       </c>
@@ -6953,11 +6968,14 @@
         <v>819</v>
       </c>
       <c r="L76" s="1"/>
+      <c r="M76" t="s">
+        <v>881</v>
+      </c>
       <c r="N76" t="s">
-        <v>882</v>
-      </c>
-    </row>
-    <row r="77" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>820</v>
       </c>
@@ -6992,11 +7010,14 @@
         <v>827</v>
       </c>
       <c r="L77" s="1"/>
+      <c r="M77" t="s">
+        <v>881</v>
+      </c>
       <c r="N77" t="s">
-        <v>882</v>
-      </c>
-    </row>
-    <row r="78" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>461</v>
       </c>
@@ -7028,13 +7049,13 @@
         <v>468</v>
       </c>
       <c r="L78" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="M78" t="s">
-        <v>1011</v>
-      </c>
-    </row>
-    <row r="79" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>469</v>
       </c>
@@ -7069,13 +7090,13 @@
         <v>475</v>
       </c>
       <c r="L79" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="M79" t="s">
-        <v>1011</v>
-      </c>
-    </row>
-    <row r="80" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>836</v>
       </c>
@@ -7107,13 +7128,13 @@
         <v>843</v>
       </c>
       <c r="L80" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="M80" t="s">
-        <v>1012</v>
-      </c>
-    </row>
-    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>851</v>
       </c>
@@ -7149,13 +7170,13 @@
         <v>857</v>
       </c>
       <c r="L81" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="M81" t="s">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="82" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>402</v>
       </c>
@@ -7193,10 +7214,10 @@
         <v>867</v>
       </c>
       <c r="M82" t="s">
-        <v>880</v>
-      </c>
-    </row>
-    <row r="83" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>582</v>
       </c>
@@ -7234,10 +7255,10 @@
         <v>867</v>
       </c>
       <c r="M83" t="s">
-        <v>881</v>
-      </c>
-    </row>
-    <row r="84" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>590</v>
       </c>
@@ -7275,10 +7296,10 @@
         <v>867</v>
       </c>
       <c r="M84" t="s">
-        <v>879</v>
-      </c>
-    </row>
-    <row r="85" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>597</v>
       </c>
@@ -7313,10 +7334,10 @@
         <v>867</v>
       </c>
       <c r="M85" t="s">
-        <v>883</v>
-      </c>
-    </row>
-    <row r="86" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>606</v>
       </c>
@@ -7354,10 +7375,10 @@
         <v>867</v>
       </c>
       <c r="M86" t="s">
-        <v>883</v>
-      </c>
-    </row>
-    <row r="87" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>612</v>
       </c>
@@ -7392,10 +7413,10 @@
         <v>867</v>
       </c>
       <c r="M87" t="s">
-        <v>884</v>
-      </c>
-    </row>
-    <row r="88" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>619</v>
       </c>
@@ -7433,10 +7454,10 @@
         <v>867</v>
       </c>
       <c r="M88" t="s">
-        <v>884</v>
-      </c>
-    </row>
-    <row r="89" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>625</v>
       </c>
@@ -7471,10 +7492,10 @@
         <v>867</v>
       </c>
       <c r="M89" t="s">
-        <v>879</v>
-      </c>
-    </row>
-    <row r="90" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>233</v>
       </c>
@@ -7506,13 +7527,13 @@
         <v>241</v>
       </c>
       <c r="L90" s="1" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="M90" t="s">
-        <v>1001</v>
-      </c>
-    </row>
-    <row r="91" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>242</v>
       </c>
@@ -7544,13 +7565,13 @@
         <v>250</v>
       </c>
       <c r="L91" s="1" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="M91" t="s">
-        <v>1001</v>
-      </c>
-    </row>
-    <row r="92" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>258</v>
       </c>
@@ -7579,13 +7600,13 @@
         <v>265</v>
       </c>
       <c r="L92" s="2" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="M92" t="s">
-        <v>1002</v>
-      </c>
-    </row>
-    <row r="93" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>719</v>
       </c>
@@ -7614,13 +7635,13 @@
         <v>725</v>
       </c>
       <c r="L93" s="4" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="M93" t="s">
-        <v>1006</v>
-      </c>
-    </row>
-    <row r="94" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>726</v>
       </c>
@@ -7652,13 +7673,13 @@
         <v>733</v>
       </c>
       <c r="L94" s="4" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="M94" t="s">
-        <v>1006</v>
-      </c>
-    </row>
-    <row r="95" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>734</v>
       </c>
@@ -7690,13 +7711,13 @@
         <v>740</v>
       </c>
       <c r="L95" s="4" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="M95" t="s">
-        <v>1006</v>
-      </c>
-    </row>
-    <row r="96" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>696</v>
       </c>
@@ -7728,13 +7749,13 @@
         <v>704</v>
       </c>
       <c r="L96" s="4" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="M96" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="97" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>712</v>
       </c>
@@ -7766,13 +7787,13 @@
         <v>718</v>
       </c>
       <c r="L97" s="4" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="M97" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="98" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>705</v>
       </c>
@@ -7804,13 +7825,13 @@
         <v>711</v>
       </c>
       <c r="L98" s="4" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="M98" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="99" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>755</v>
       </c>
@@ -7839,13 +7860,13 @@
         <v>762</v>
       </c>
       <c r="L99" s="4" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="M99" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="100" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>763</v>
       </c>
@@ -7877,13 +7898,13 @@
         <v>770</v>
       </c>
       <c r="L100" s="4" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="M100" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="101" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>771</v>
       </c>
@@ -7912,13 +7933,13 @@
         <v>778</v>
       </c>
       <c r="L101" s="3" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="M101" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="102" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>426</v>
       </c>
@@ -7953,13 +7974,13 @@
         <v>432</v>
       </c>
       <c r="L102" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="M102" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="103" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>433</v>
       </c>
@@ -7994,13 +8015,13 @@
         <v>440</v>
       </c>
       <c r="L103" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="M103" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="104" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>418</v>
       </c>
@@ -8035,13 +8056,13 @@
         <v>425</v>
       </c>
       <c r="L104" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="M104" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="105" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>561</v>
       </c>
@@ -8076,13 +8097,13 @@
         <v>567</v>
       </c>
       <c r="L105" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="M105" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="106" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>568</v>
       </c>
@@ -8118,13 +8139,13 @@
         <v>574</v>
       </c>
       <c r="L106" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="M106" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="107" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>554</v>
       </c>
@@ -8159,13 +8180,13 @@
         <v>560</v>
       </c>
       <c r="L107" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="M107" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="108" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>190</v>
       </c>
@@ -8194,13 +8215,13 @@
         <v>196</v>
       </c>
       <c r="L108" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="M108" t="s">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="109" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>369</v>
       </c>
@@ -8232,13 +8253,13 @@
         <v>376</v>
       </c>
       <c r="L109" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="M109" t="s">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="110" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>410</v>
       </c>
@@ -8273,13 +8294,13 @@
         <v>417</v>
       </c>
       <c r="L110" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="M110" t="s">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="111" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>741</v>
       </c>
@@ -8314,16 +8335,16 @@
         <v>748</v>
       </c>
       <c r="L111" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="M111" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="N111" t="s">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="112" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>749</v>
       </c>
@@ -8358,16 +8379,16 @@
         <v>748</v>
       </c>
       <c r="L112" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="M112" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="N112" t="s">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="113" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>98</v>
       </c>
@@ -8399,16 +8420,16 @@
         <v>105</v>
       </c>
       <c r="L113" s="1" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="M113" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="N113" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="114" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>251</v>
       </c>
@@ -8441,13 +8462,13 @@
         <v>257</v>
       </c>
       <c r="L114" s="1" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="M114" t="s">
+        <v>1003</v>
+      </c>
+      <c r="N114" t="s">
         <v>1004</v>
-      </c>
-      <c r="N114" t="s">
-        <v>1005</v>
       </c>
     </row>
   </sheetData>
@@ -8469,458 +8490,458 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>995</v>
+      </c>
+      <c r="B1" t="s">
         <v>996</v>
-      </c>
-      <c r="B1" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>884</v>
+      </c>
+      <c r="B2" t="s">
         <v>885</v>
-      </c>
-      <c r="B2" t="s">
-        <v>886</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>886</v>
+      </c>
+      <c r="B3" t="s">
         <v>887</v>
-      </c>
-      <c r="B3" t="s">
-        <v>888</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>888</v>
+      </c>
+      <c r="B4" t="s">
         <v>889</v>
-      </c>
-      <c r="B4" t="s">
-        <v>890</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>890</v>
+      </c>
+      <c r="B5" t="s">
         <v>891</v>
-      </c>
-      <c r="B5" t="s">
-        <v>892</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>892</v>
+      </c>
+      <c r="B6" t="s">
         <v>893</v>
-      </c>
-      <c r="B6" t="s">
-        <v>894</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>894</v>
+      </c>
+      <c r="B7" t="s">
         <v>895</v>
-      </c>
-      <c r="B7" t="s">
-        <v>896</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>896</v>
+      </c>
+      <c r="B8" t="s">
         <v>897</v>
-      </c>
-      <c r="B8" t="s">
-        <v>898</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>898</v>
+      </c>
+      <c r="B9" t="s">
         <v>899</v>
-      </c>
-      <c r="B9" t="s">
-        <v>900</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>900</v>
+      </c>
+      <c r="B10" t="s">
         <v>901</v>
-      </c>
-      <c r="B10" t="s">
-        <v>902</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>902</v>
+      </c>
+      <c r="B11" t="s">
         <v>903</v>
-      </c>
-      <c r="B11" t="s">
-        <v>904</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>904</v>
+      </c>
+      <c r="B12" t="s">
         <v>905</v>
-      </c>
-      <c r="B12" t="s">
-        <v>906</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>906</v>
+      </c>
+      <c r="B13" t="s">
         <v>907</v>
-      </c>
-      <c r="B13" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>908</v>
+      </c>
+      <c r="B14" t="s">
         <v>909</v>
-      </c>
-      <c r="B14" t="s">
-        <v>910</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>910</v>
+      </c>
+      <c r="B15" t="s">
         <v>911</v>
-      </c>
-      <c r="B15" t="s">
-        <v>912</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>912</v>
+      </c>
+      <c r="B16" t="s">
         <v>913</v>
-      </c>
-      <c r="B16" t="s">
-        <v>914</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>914</v>
+      </c>
+      <c r="B17" t="s">
         <v>915</v>
-      </c>
-      <c r="B17" t="s">
-        <v>916</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>916</v>
+      </c>
+      <c r="B18" t="s">
         <v>917</v>
-      </c>
-      <c r="B18" t="s">
-        <v>918</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>918</v>
+      </c>
+      <c r="B19" t="s">
         <v>919</v>
-      </c>
-      <c r="B19" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>920</v>
+      </c>
+      <c r="B20" t="s">
         <v>921</v>
-      </c>
-      <c r="B20" t="s">
-        <v>922</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>922</v>
+      </c>
+      <c r="B21" t="s">
         <v>923</v>
-      </c>
-      <c r="B21" t="s">
-        <v>924</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>924</v>
+      </c>
+      <c r="B22" t="s">
         <v>925</v>
-      </c>
-      <c r="B22" t="s">
-        <v>926</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>926</v>
+      </c>
+      <c r="B23" t="s">
         <v>927</v>
-      </c>
-      <c r="B23" t="s">
-        <v>928</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>928</v>
+      </c>
+      <c r="B24" t="s">
         <v>929</v>
-      </c>
-      <c r="B24" t="s">
-        <v>930</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>930</v>
+      </c>
+      <c r="B25" t="s">
         <v>931</v>
-      </c>
-      <c r="B25" t="s">
-        <v>932</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>932</v>
+      </c>
+      <c r="B26" t="s">
         <v>933</v>
-      </c>
-      <c r="B26" t="s">
-        <v>934</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>934</v>
+      </c>
+      <c r="B27" t="s">
         <v>935</v>
-      </c>
-      <c r="B27" t="s">
-        <v>936</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>936</v>
+      </c>
+      <c r="B28" t="s">
         <v>937</v>
-      </c>
-      <c r="B28" t="s">
-        <v>938</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>938</v>
+      </c>
+      <c r="B29" t="s">
         <v>939</v>
-      </c>
-      <c r="B29" t="s">
-        <v>940</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>940</v>
+      </c>
+      <c r="B30" t="s">
         <v>941</v>
-      </c>
-      <c r="B30" t="s">
-        <v>942</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>942</v>
+      </c>
+      <c r="B31" t="s">
         <v>943</v>
-      </c>
-      <c r="B31" t="s">
-        <v>944</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>944</v>
+      </c>
+      <c r="B32" t="s">
         <v>945</v>
-      </c>
-      <c r="B32" t="s">
-        <v>946</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>946</v>
+      </c>
+      <c r="B33" t="s">
         <v>947</v>
-      </c>
-      <c r="B33" t="s">
-        <v>948</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>948</v>
+      </c>
+      <c r="B34" t="s">
         <v>949</v>
-      </c>
-      <c r="B34" t="s">
-        <v>950</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>950</v>
+      </c>
+      <c r="B35" t="s">
         <v>951</v>
-      </c>
-      <c r="B35" t="s">
-        <v>952</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>952</v>
+      </c>
+      <c r="B36" t="s">
         <v>953</v>
-      </c>
-      <c r="B36" t="s">
-        <v>954</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>954</v>
+      </c>
+      <c r="B37" t="s">
         <v>955</v>
-      </c>
-      <c r="B37" t="s">
-        <v>956</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>956</v>
+      </c>
+      <c r="B38" t="s">
         <v>957</v>
-      </c>
-      <c r="B38" t="s">
-        <v>958</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>958</v>
+      </c>
+      <c r="B39" t="s">
         <v>959</v>
-      </c>
-      <c r="B39" t="s">
-        <v>960</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>960</v>
+      </c>
+      <c r="B40" t="s">
         <v>961</v>
-      </c>
-      <c r="B40" t="s">
-        <v>962</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>962</v>
+      </c>
+      <c r="B41" t="s">
         <v>963</v>
-      </c>
-      <c r="B41" t="s">
-        <v>964</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>964</v>
+      </c>
+      <c r="B42" t="s">
         <v>965</v>
-      </c>
-      <c r="B42" t="s">
-        <v>966</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>966</v>
+      </c>
+      <c r="B43" t="s">
         <v>967</v>
-      </c>
-      <c r="B43" t="s">
-        <v>968</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>968</v>
+      </c>
+      <c r="B44" t="s">
         <v>969</v>
-      </c>
-      <c r="B44" t="s">
-        <v>970</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>970</v>
+      </c>
+      <c r="B45" t="s">
         <v>971</v>
-      </c>
-      <c r="B45" t="s">
-        <v>972</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>972</v>
+      </c>
+      <c r="B46" t="s">
         <v>973</v>
-      </c>
-      <c r="B46" t="s">
-        <v>974</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>974</v>
+      </c>
+      <c r="B47" t="s">
         <v>975</v>
-      </c>
-      <c r="B47" t="s">
-        <v>976</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>976</v>
+      </c>
+      <c r="B48" t="s">
         <v>977</v>
-      </c>
-      <c r="B48" t="s">
-        <v>978</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>978</v>
+      </c>
+      <c r="B49" t="s">
         <v>979</v>
-      </c>
-      <c r="B49" t="s">
-        <v>980</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>980</v>
+      </c>
+      <c r="B50" t="s">
         <v>981</v>
-      </c>
-      <c r="B50" t="s">
-        <v>982</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>982</v>
+      </c>
+      <c r="B51" t="s">
         <v>983</v>
-      </c>
-      <c r="B51" t="s">
-        <v>984</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>984</v>
+      </c>
+      <c r="B52" t="s">
         <v>985</v>
-      </c>
-      <c r="B52" t="s">
-        <v>986</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
+        <v>986</v>
+      </c>
+      <c r="B53" t="s">
         <v>987</v>
-      </c>
-      <c r="B53" t="s">
-        <v>988</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B54" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>989</v>
+      </c>
+      <c r="B55" t="s">
         <v>990</v>
-      </c>
-      <c r="B55" t="s">
-        <v>991</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>991</v>
+      </c>
+      <c r="B56" t="s">
         <v>992</v>
-      </c>
-      <c r="B56" t="s">
-        <v>993</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
+        <v>993</v>
+      </c>
+      <c r="B57" t="s">
         <v>994</v>
-      </c>
-      <c r="B57" t="s">
-        <v>995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>